<commit_message>
Implement reporting bible and objective gates
</commit_message>
<xml_diff>
--- a/outputs/commercial-quality/essential-supporting-register.xlsx
+++ b/outputs/commercial-quality/essential-supporting-register.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R5e8a5cdebb5b48eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="Rb1160ab1fdc84094"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="3" r:id="R753778972e1b455e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Actions" sheetId="4" r:id="R8f47449f36754f82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Checklist" sheetId="5" r:id="R42bb644f1eda4e74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" r:id="R379f53cd375d4e2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Trace" sheetId="7" r:id="Rbb120915ea324443"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Improvements" sheetId="8" r:id="R38257009eb9147e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R5241328da710499c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="Rb230e4c0c922441f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="3" r:id="R041581376e184fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Actions" sheetId="4" r:id="R155b5612ce1f46f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Checklist" sheetId="5" r:id="R9301ac75756c4c7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" r:id="R8d7c8a6ab5d04a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Trace" sheetId="7" r:id="R3520ca58f2ab4b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Improvements" sheetId="8" r:id="Ra8f6bd157d5248c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -517,7 +517,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04fe82469b794308"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dda75f9b7444d55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2509,7 +2509,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra056ea4b0674492d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1920e5eb0714d1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3848,7 +3848,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3402c2b29fd24acf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75ea49e41eaa4c31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5840,7 +5840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf23b700763bf4c05"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98697fc7759d42b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9998,7 +9998,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72d8e7a79a5f4e76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1dafc1d9cf74bf2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11292,7 +11292,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bb2c9c33b774ebc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b4c90c812b147d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13832,7 +13832,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d63cc34a06a46c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81acb31561054a49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14870,7 +14870,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc674525afc4c4f67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R749f6187bccd4744"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct Comprehensive Reporting Bible architecture
</commit_message>
<xml_diff>
--- a/outputs/commercial-quality/essential-supporting-register.xlsx
+++ b/outputs/commercial-quality/essential-supporting-register.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R5241328da710499c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="Rb230e4c0c922441f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="3" r:id="R041581376e184fe9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Actions" sheetId="4" r:id="R155b5612ce1f46f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Checklist" sheetId="5" r:id="R9301ac75756c4c7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" r:id="R8d7c8a6ab5d04a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Trace" sheetId="7" r:id="R3520ca58f2ab4b82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Improvements" sheetId="8" r:id="Ra8f6bd157d5248c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" r:id="R7c514e3da6664cb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R36bfd850879c4ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="3" r:id="R9a985ee5bef846b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Actions" sheetId="4" r:id="Ra26a7b6e11ce4026"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Checklist" sheetId="5" r:id="Read80b8cab454de8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" r:id="Re847b2e796b1421b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Trace" sheetId="7" r:id="R8ea3bca6c2244683"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Improvements" sheetId="8" r:id="R6b05ba5ef9684d02"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -517,7 +517,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7dda75f9b7444d55"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce6dedf4112e4967"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2509,7 +2509,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1920e5eb0714d1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f1729617c124211"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3848,7 +3848,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75ea49e41eaa4c31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebc615a9e6764bb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5840,7 +5840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98697fc7759d42b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4cdc2a45d914c47"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9998,7 +9998,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1dafc1d9cf74bf2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1da3875327344545"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11292,7 +11292,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b4c90c812b147d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65aa65fad6b54675"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13832,7 +13832,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81acb31561054a49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64554d1681e44e3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14870,7 +14870,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R749f6187bccd4744"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae5192ddd5d54cfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>